<commit_message>
scan: seg4 2026-07-01 20:38 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-07-01.xlsx
+++ b/output/full_scan/batch_seq5_2026-07-01.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -686,21 +686,21 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>4763</v>
+        <v>6141</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>材料*-KY</t>
+          <t>柏承</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v/>
       </c>
       <c r="D5" s="2" t="n">
-        <v>656.9627667384968</v>
+        <v>691.7678795534702</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>47.9</v>
+        <v>39.3</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -711,13 +711,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>62.06212574615586</v>
+        <v>56.74182875236681</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>20.65422806843356</v>
+        <v>20.03462519542085</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>1.699092286072959</v>
+        <v>0.3264345735128945</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>0</v>
@@ -729,31 +729,31 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.2968938591378667</v>
+        <v>0.2082601449531487</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5519</v>
+        <v>4763</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>隆大</t>
+          <t>材料*-KY</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v/>
       </c>
       <c r="D6" s="2" t="n">
-        <v>634.3364083431576</v>
+        <v>656.9627667384968</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>34.5</v>
+        <v>47.9</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -764,13 +764,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>61.29759807213868</v>
+        <v>62.06212574615586</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>27.50219288655432</v>
+        <v>20.65422806843356</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>0.6804179686561578</v>
+        <v>1.699092286072959</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>0</v>
@@ -782,31 +782,31 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.0316388582012249</v>
+        <v>0.2968938591378667</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, bb_squeeze_breakout, breakout_volume_confirm, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>6156</v>
+        <v>5519</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>松上</t>
+          <t>隆大</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>620.5843988038382</v>
+        <v>634.3364083431576</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>31.65</v>
+        <v>34.5</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -817,13 +817,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>80.36041522377478</v>
+        <v>61.29759807213868</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>40.79651259303245</v>
+        <v>27.50219288655432</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>1.158439880383816</v>
+        <v>0.6804179686561578</v>
       </c>
       <c r="K7" s="2" t="n">
         <v>0</v>
@@ -835,31 +835,31 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.7558276987277435</v>
+        <v>0.0316388582012249</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6138</v>
+        <v>6156</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>茂達</t>
+          <t>松上</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>620.26402155825</v>
+        <v>620.5843988038382</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>380.5</v>
+        <v>31.65</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,13 +870,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>60.97098365835977</v>
+        <v>80.36041522377478</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>22.02202201371272</v>
+        <v>40.79651259303245</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2.655184858547434</v>
+        <v>1.158439880383816</v>
       </c>
       <c r="K8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.994202231534061</v>
+        <v>0.7558276987277435</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6129</v>
+        <v>6138</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>普誠</t>
+          <t>茂達</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>618.6617854286051</v>
+        <v>620.26402155825</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>18.3</v>
+        <v>380.5</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>60.50357637864965</v>
+        <v>60.97098365835977</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>25.11538495569169</v>
+        <v>22.02202201371272</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>0.7127443325971251</v>
+        <v>2.655184858547434</v>
       </c>
       <c r="K9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.2325116567405371</v>
+        <v>1.994202231534061</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>4564</v>
+        <v>6129</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>元翎</t>
+          <t>普誠</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>613.5003821335728</v>
+        <v>618.6617854286051</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>16.25</v>
+        <v>18.3</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,13 +976,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>54.80900555566682</v>
+        <v>60.50357637864965</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>27.43147056569617</v>
+        <v>25.11538495569169</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>2.757611991813016</v>
+        <v>0.7127443325971251</v>
       </c>
       <c r="K10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.1306409949661282</v>
+        <v>0.2325116567405371</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>4306</v>
+        <v>4564</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>炎洲</t>
+          <t>元翎</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>611.8867260687252</v>
+        <v>613.5003821335728</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>15.9</v>
+        <v>16.25</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>68.92721512762466</v>
+        <v>54.80900555566682</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>42.00849214319383</v>
+        <v>27.43147056569617</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>0.5392861730970653</v>
+        <v>2.757611991813016</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.06867287653171</v>
+        <v>0.1306409949661282</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>4536</v>
+        <v>4306</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>拓凱</t>
+          <t>炎洲</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>580.2216144085183</v>
+        <v>611.8867260687252</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>167.5</v>
+        <v>15.9</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63.90168703186922</v>
+        <v>68.92721512762466</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>21.22357150616251</v>
+        <v>42.00849214319383</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>1.105020117909853</v>
+        <v>0.5392861730970653</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.0387869296918244</v>
+        <v>-0.06867287653171</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>4722</v>
+        <v>4551</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>國精化</t>
+          <t>智伸科</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>577.3699823935581</v>
+        <v>606.1573506903392</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>275.5</v>
+        <v>234</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>52.94636630339669</v>
+        <v>71.12563583029092</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>29.96278122105414</v>
+        <v>37.66652200697235</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>0.7018155478942868</v>
+        <v>0.4139097522792758</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>1.442812551504591</v>
+        <v>3.291990676372038</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>4590</v>
+        <v>4536</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>富田-創</t>
+          <t>拓凱</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>576.6328437327085</v>
+        <v>580.2216144085183</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>80</v>
+        <v>167.5</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.45765952521945</v>
+        <v>63.90168703186922</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>15.55429026865683</v>
+        <v>21.22357150616251</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1.819195018086909</v>
+        <v>1.105020117909853</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.2182722881251616</v>
+        <v>-0.0387869296918244</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6024</v>
+        <v>4722</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>群益期</t>
+          <t>國精化</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>565.630713763813</v>
+        <v>577.3699823935581</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>61.7</v>
+        <v>275.5</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>61.24576022300645</v>
+        <v>52.94636630339669</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>25.06334294742515</v>
+        <v>29.96278122105414</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.344816767927841</v>
+        <v>0.7018155478942868</v>
       </c>
       <c r="K15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>-0.1800298069673451</v>
+        <v>1.442812551504591</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>5288</v>
+        <v>4590</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>豐祥-KY</t>
+          <t>富田-創</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>502.9725723262133</v>
+        <v>576.6328437327085</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>178.5</v>
+        <v>80</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,13 +1294,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>54.37799066473929</v>
+        <v>60.45765952521945</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>24.07411670227109</v>
+        <v>15.55429026865683</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.8994588347597756</v>
+        <v>1.819195018086909</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-1.608440480286304</v>
+        <v>0.2182722881251616</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>5876</v>
+        <v>6024</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>上海商銀</t>
+          <t>群益期</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>502.387638992861</v>
+        <v>565.630713763813</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>42.4</v>
+        <v>61.7</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,13 +1347,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>57.55367445726819</v>
+        <v>61.24576022300645</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>26.79922103966467</v>
+        <v>25.06334294742515</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>0.451580489418335</v>
+        <v>0.344816767927841</v>
       </c>
       <c r="K17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-0.0237912802851255</v>
+        <v>-0.1800298069673451</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>4526</v>
+        <v>4764</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>東台</t>
+          <t>雙鍵</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>496.3379553427016</v>
+        <v>563.3054202238948</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>41.15</v>
+        <v>301</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,16 +1400,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>53.70804067122585</v>
+        <v>51.16597962896741</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>24.57449692907823</v>
+        <v>15.84811932720879</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1.453133942795667</v>
+        <v>0.1868041908960731</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-0.0637794289063851</v>
+        <v>-2.066855240572797</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6154</v>
+        <v>5288</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>順發</t>
+          <t>豐祥-KY</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>493.6032669879718</v>
+        <v>502.9725723262133</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>13.75</v>
+        <v>178.5</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>51.18062085101813</v>
+        <v>54.37799066473929</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.28637081244341</v>
+        <v>24.07411670227109</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>0.2740033248203728</v>
+        <v>0.8994588347597756</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.042475720466533</v>
+        <v>-1.608440480286304</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>4439</v>
+        <v>5876</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>冠星-KY</t>
+          <t>上海商銀</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>492.2663210890062</v>
+        <v>502.387638992861</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>42.4</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>50.45932615382573</v>
+        <v>57.55367445726819</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.52228051977085</v>
+        <v>26.79922103966467</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.652028518124389</v>
+        <v>0.451580489418335</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.3301895959381894</v>
+        <v>-0.0237912802851255</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6134</v>
+        <v>4526</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>萬旭</t>
+          <t>東台</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>490.9192124190721</v>
+        <v>496.3379553427016</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>34.05</v>
+        <v>41.15</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,13 +1559,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>48.68594802620877</v>
+        <v>53.70804067122585</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>11.22378550709127</v>
+        <v>24.57449692907823</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>0.6110125416396927</v>
+        <v>1.453133942795667</v>
       </c>
       <c r="K21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.2455209776984779</v>
+        <v>-0.0637794289063851</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>4576</v>
+        <v>6154</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>大銀微系統</t>
+          <t>順發</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>489.6966632778364</v>
+        <v>493.6032669879718</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>214</v>
+        <v>13.75</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>47.68090553668037</v>
+        <v>51.18062085101813</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21.52347688535022</v>
+        <v>23.28637081244341</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.9245516470069784</v>
+        <v>0.2740033248203728</v>
       </c>
       <c r="K22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-0.5909936021814444</v>
+        <v>-0.042475720466533</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6005</v>
+        <v>4439</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>群益證</t>
+          <t>冠星-KY</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>452.3652215410151</v>
+        <v>492.2663210890062</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>37.65</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,13 +1665,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>49.42998841126707</v>
+        <v>50.45932615382573</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>34.54682023778955</v>
+        <v>32.52228051977085</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>0.5041893128042311</v>
+        <v>0.652028518124389</v>
       </c>
       <c r="K23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.601622376812716</v>
+        <v>0.3301895959381894</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>4572</v>
+        <v>6134</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>駐龍</t>
+          <t>萬旭</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>450.970061540788</v>
+        <v>490.9192124190721</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>146</v>
+        <v>34.05</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,13 +1718,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>54.45562478390875</v>
+        <v>48.68594802620877</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>17.25098787911467</v>
+        <v>11.22378550709127</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1.135285062476597</v>
+        <v>0.6110125416396927</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.050026287220765</v>
+        <v>-0.2455209776984779</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6147</v>
+        <v>4576</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>頎邦</t>
+          <t>大銀微系統</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>442.714773932907</v>
+        <v>489.6966632778364</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1771,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>45.80251755276391</v>
+        <v>47.68090553668037</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>24.4532736557268</v>
+        <v>21.52347688535022</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>1.181464796643528</v>
+        <v>0.9245516470069784</v>
       </c>
       <c r="K25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-6.693629003511619</v>
+        <v>-0.5909936021814444</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>5534</v>
+        <v>6005</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>長虹</t>
+          <t>群益證</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>437.4305346702486</v>
+        <v>452.3652215410151</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>79</v>
+        <v>37.65</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,13 +1824,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>50.35866187861998</v>
+        <v>49.42998841126707</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.69267971272414</v>
+        <v>34.54682023778955</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.235974954943801</v>
+        <v>0.5041893128042311</v>
       </c>
       <c r="K26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>-0.3593740178706665</v>
+        <v>-0.601622376812716</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>5306</v>
+        <v>4572</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>桂盟</t>
+          <t>駐龍</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>431.3310997468327</v>
+        <v>450.970061540788</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>85.8</v>
+        <v>146</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>53.0128978033806</v>
+        <v>54.45562478390875</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>22.91566382122724</v>
+        <v>17.25098787911467</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.2969515194115791</v>
+        <v>1.135285062476597</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-0.1476297835614404</v>
+        <v>0.050026287220765</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>4720</v>
+        <v>6147</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>德淵</t>
+          <t>頎邦</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>425.0516203405547</v>
+        <v>442.714773932907</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>24.15</v>
+        <v>219</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>48.22772343335434</v>
+        <v>45.80251755276391</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>14.54483442521492</v>
+        <v>24.4532736557268</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.6209275404502775</v>
+        <v>1.181464796643528</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.0183493395429201</v>
+        <v>-6.693629003511619</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6161</v>
+        <v>5534</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>捷波</t>
+          <t>長虹</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>421.6716567962322</v>
+        <v>437.4305346702486</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>52.4</v>
+        <v>79</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>50.86740121011348</v>
+        <v>50.35866187861998</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>14.59666588280698</v>
+        <v>23.69267971272414</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.6469603805806211</v>
+        <v>0.235974954943801</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-0.4759777755828455</v>
+        <v>-0.3593740178706665</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>5284</v>
+        <v>5306</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>jpp-KY</t>
+          <t>桂盟</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>415.0113934528406</v>
+        <v>431.3310997468327</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>373.5</v>
+        <v>85.8</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>46.8500330997596</v>
+        <v>53.0128978033806</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18.51972773996315</v>
+        <v>22.91566382122724</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.958031154170944</v>
+        <v>0.2969515194115791</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-2.563316193656069</v>
+        <v>-0.1476297835614404</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>4739</v>
+        <v>4720</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>康普</t>
+          <t>德淵</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>414.4672677927212</v>
+        <v>425.0516203405547</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>111.5</v>
+        <v>24.15</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>48.79736218577888</v>
+        <v>48.22772343335434</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>21.89114092197599</v>
+        <v>14.54483442521492</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>0.430122127742635</v>
+        <v>0.6209275404502775</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-2.382085251121663</v>
+        <v>0.0183493395429201</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>4771</v>
+        <v>6161</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>望隼</t>
+          <t>捷波</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>410.7064142020189</v>
+        <v>421.6716567962322</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>195.5</v>
+        <v>52.4</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,13 +2142,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.53037901300222</v>
+        <v>50.86740121011348</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>13.09328640829183</v>
+        <v>14.59666588280698</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.9237577601994392</v>
+        <v>0.6469603805806211</v>
       </c>
       <c r="K32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.4164772007109762</v>
+        <v>-0.4759777755828455</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6163</v>
+        <v>5284</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>華電網</t>
+          <t>jpp-KY</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>396.5713048835844</v>
+        <v>415.0113934528406</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>48.7</v>
+        <v>373.5</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>42.87944494723448</v>
+        <v>46.8500330997596</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>19.63301548148938</v>
+        <v>18.51972773996315</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.3112967664630154</v>
+        <v>0.958031154170944</v>
       </c>
       <c r="K33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.0075760515269824</v>
+        <v>-2.563316193656069</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>4807</v>
+        <v>4739</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>日成-KY</t>
+          <t>康普</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>392.0164974300798</v>
+        <v>414.4672677927212</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>37.55</v>
+        <v>111.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,13 +2248,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.29659105999149</v>
+        <v>48.79736218577888</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>50.69094966785645</v>
+        <v>21.89114092197599</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.3670452854521105</v>
+        <v>0.430122127742635</v>
       </c>
       <c r="K34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-1.150789969266585</v>
+        <v>-2.382085251121663</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>4746</v>
+        <v>4771</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>台耀</t>
+          <t>望隼</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>389.4127823395181</v>
+        <v>410.7064142020189</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>53.7</v>
+        <v>195.5</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,13 +2301,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>56.29586590381918</v>
+        <v>55.53037901300222</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>8.707170963410102</v>
+        <v>13.09328640829183</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.655410434122415</v>
+        <v>0.9237577601994392</v>
       </c>
       <c r="K35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.2444131339717775</v>
+        <v>0.4164772007109762</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6143</v>
+        <v>6163</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>振曜</t>
+          <t>華電網</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>387.1708270674019</v>
+        <v>396.5713048835844</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>93.40000000000001</v>
+        <v>48.7</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,13 +2354,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>52.54425905116103</v>
+        <v>42.87944494723448</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>22.06998349528193</v>
+        <v>19.63301548148938</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.8342738101005832</v>
+        <v>0.3112967664630154</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.5317882717492008</v>
+        <v>0.0075760515269824</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>4581</v>
+        <v>4807</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>光隆精密-KY</t>
+          <t>日成-KY</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>378.8005699769136</v>
+        <v>392.0164974300798</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>50.1</v>
+        <v>37.55</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,13 +2407,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>52.04105032065947</v>
+        <v>54.29659105999149</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>14.01645626955793</v>
+        <v>50.69094966785645</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>1.103275947599537</v>
+        <v>0.3670452854521105</v>
       </c>
       <c r="K37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.2545723081623134</v>
+        <v>-1.150789969266585</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>5522</v>
+        <v>4746</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>遠雄</t>
+          <t>台耀</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>369.2277485455275</v>
+        <v>389.4127823395181</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>64.59999999999999</v>
+        <v>53.7</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>31.53556210421356</v>
+        <v>56.29586590381918</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>27.73164359088942</v>
+        <v>8.707170963410102</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.122774854552752</v>
+        <v>1.655410434122415</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-1.532877418231151</v>
+        <v>0.2444131339717775</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>4555</v>
+        <v>6143</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>氣立</t>
+          <t>振曜</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>365.4158114124792</v>
+        <v>387.1708270674019</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>48.8</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,13 +2513,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>53.00686274130292</v>
+        <v>52.54425905116103</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>19.78383446274585</v>
+        <v>22.06998349528193</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.9263574148124883</v>
+        <v>0.8342738101005832</v>
       </c>
       <c r="K39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.2239356482760417</v>
+        <v>0.5317882717492008</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>5538</v>
+        <v>4581</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>東明-KY</t>
+          <t>光隆精密-KY</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>356.6061450653635</v>
+        <v>378.8005699769136</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>32.85</v>
+        <v>50.1</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>49.25428964234276</v>
+        <v>52.04105032065947</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>16.84079937190634</v>
+        <v>14.01645626955793</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.1324510972518607</v>
+        <v>1.103275947599537</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.0145740028082888</v>
+        <v>0.2545723081623134</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6146</v>
+        <v>5522</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>耕興</t>
+          <t>遠雄</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>356.5892164551082</v>
+        <v>369.2277485455275</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>191</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,13 +2619,13 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>35.90712230891251</v>
+        <v>31.53556210421356</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>33.13207304912729</v>
+        <v>27.73164359088942</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.6105682452894078</v>
+        <v>1.122774854552752</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.4797692771530188</v>
+        <v>-1.532877418231151</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2647,21 +2647,21 @@
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>5283</v>
+        <v>4555</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>禾聯碩</t>
+          <t>氣立</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>356.34546633505</v>
+        <v>365.4158114124792</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>52.7</v>
+        <v>48.8</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,13 +2672,13 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>45.6196709769978</v>
+        <v>53.00686274130292</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>22.34505584603467</v>
+        <v>19.78383446274585</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.6101537390871262</v>
+        <v>0.9263574148124883</v>
       </c>
       <c r="K42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.1676582301808917</v>
+        <v>-0.2239356482760417</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>4569</v>
+        <v>5538</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>六方科-KY</t>
+          <t>東明-KY</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>352.4109544321478</v>
+        <v>356.6061450653635</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>173</v>
+        <v>32.85</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,13 +2725,13 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>48.54815263454783</v>
+        <v>49.25428964234276</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>13.30117959782311</v>
+        <v>16.84079937190634</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.596205593389581</v>
+        <v>0.1324510972518607</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>0</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.637784841685632</v>
+        <v>-0.0145740028082888</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2753,21 +2753,21 @@
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>4571</v>
+        <v>6146</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>鈞興-KY</t>
+          <t>耕興</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>341.378154747154</v>
+        <v>356.5892164551082</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,13 +2778,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>36.44098546517739</v>
+        <v>35.90712230891251</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>30.13329255380932</v>
+        <v>33.13207304912729</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.4690436222484413</v>
+        <v>0.6105682452894078</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>0</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-1.625009955750815</v>
+        <v>-0.4797692771530188</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2806,21 +2806,21 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>4560</v>
+        <v>5283</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>強信-KY</t>
+          <t>禾聯碩</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>337.7729274683856</v>
+        <v>356.34546633505</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>33.05</v>
+        <v>52.7</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>52.21666819138976</v>
+        <v>45.6196709769978</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>18.18411079027799</v>
+        <v>22.34505584603467</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>1.40751482128406</v>
+        <v>0.6101537390871262</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.1072236905983305</v>
+        <v>-0.1676582301808917</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>4755</v>
+        <v>4569</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>三福化</t>
+          <t>六方科-KY</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>335.3594691915536</v>
+        <v>352.4109544321478</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>128.5</v>
+        <v>173</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,13 +2884,13 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>37.22409159286018</v>
+        <v>48.54815263454783</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>14.74969617090118</v>
+        <v>13.30117959782311</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>2.256267134262167</v>
+        <v>0.596205593389581</v>
       </c>
       <c r="K46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-1.094428985326426</v>
+        <v>-0.637784841685632</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>5871</v>
+        <v>4571</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>中租-KY</t>
+          <t>鈞興-KY</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>335.3263777083471</v>
+        <v>341.378154747154</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>114.5</v>
+        <v>168</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>48.93513756555246</v>
+        <v>36.44098546517739</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>11.70236717603665</v>
+        <v>30.13329255380932</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.6405362883123391</v>
+        <v>0.4690436222484413</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.3717589066432479</v>
+        <v>-1.625009955750815</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>4737</v>
+        <v>4560</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>華廣</t>
+          <t>強信-KY</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>322.0380443627744</v>
+        <v>337.7729274683856</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>57.2</v>
+        <v>33.05</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>51.74495917014591</v>
+        <v>52.21666819138976</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>14.75604033963378</v>
+        <v>18.18411079027799</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>1.180619275220998</v>
+        <v>1.40751482128406</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.2738690139160426</v>
+        <v>0.1072236905983305</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>4190</v>
+        <v>4755</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>佐登-KY</t>
+          <t>三福化</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>318.1860196504719</v>
+        <v>335.3594691915536</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>25</v>
+        <v>128.5</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.16033230340451</v>
+        <v>37.22409159286018</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>27.42493312644127</v>
+        <v>14.74969617090118</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.6794658859518247</v>
+        <v>2.256267134262167</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.07008943232299041</v>
+        <v>-1.094428985326426</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>5607</v>
+        <v>5871</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>遠雄港</t>
+          <t>中租-KY</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>307.5514588926027</v>
+        <v>335.3263777083471</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>50.2</v>
+        <v>114.5</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>44.55506969970366</v>
+        <v>48.93513756555246</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>16.42997910994498</v>
+        <v>11.70236717603665</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.5123282204167089</v>
+        <v>0.6405362883123391</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.3246707904279218</v>
+        <v>-0.3717589066432479</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>5525</v>
+        <v>4737</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>順天</t>
+          <t>華廣</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>305.5250611701271</v>
+        <v>322.0380443627744</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>21.6</v>
+        <v>57.2</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>42.67387788355755</v>
+        <v>51.74495917014591</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.32391687742012</v>
+        <v>14.75604033963378</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.9789328400564156</v>
+        <v>1.180619275220998</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.0155094942503423</v>
+        <v>0.2738690139160426</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>5546</v>
+        <v>4190</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>永固-KY</t>
+          <t>佐登-KY</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>305.1420126710896</v>
+        <v>318.1860196504719</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>16.3</v>
+        <v>25</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,13 +3202,13 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>46.71841238260079</v>
+        <v>53.16033230340451</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>31.99837793131048</v>
+        <v>27.42493312644127</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.0273962157990979</v>
+        <v>0.6794658859518247</v>
       </c>
       <c r="K52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.0609011067201433</v>
+        <v>0.07008943232299041</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>4414</v>
+        <v>5607</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>如興</t>
+          <t>遠雄港</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>303.0777965631694</v>
+        <v>307.5514588926027</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>8.470000000000001</v>
+        <v>50.2</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,13 +3255,13 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>46.29764193570838</v>
+        <v>44.55506969970366</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>16.83253887990648</v>
+        <v>16.42997910994498</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.4623435669650748</v>
+        <v>0.5123282204167089</v>
       </c>
       <c r="K53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.06304644204970471</v>
+        <v>-0.3246707904279218</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>4583</v>
+        <v>5525</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>台灣精銳</t>
+          <t>順天</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>291.0945889811774</v>
+        <v>305.5250611701271</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>605</v>
+        <v>21.6</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>38.27581033002252</v>
+        <v>42.67387788355755</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>36.05056018009433</v>
+        <v>19.32391687742012</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.9339098843506094</v>
+        <v>0.9789328400564156</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.4191200266180388</v>
+        <v>-0.0155094942503423</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>4766</v>
+        <v>5546</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>南寶</t>
+          <t>永固-KY</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>275.5298205404143</v>
+        <v>305.1420126710896</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>356.5</v>
+        <v>16.3</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,13 +3361,13 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>48.66618856689502</v>
+        <v>46.71841238260079</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>16.95375094222679</v>
+        <v>31.99837793131048</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1.068839097627098</v>
+        <v>0.0273962157990979</v>
       </c>
       <c r="K55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-2.089189099028857</v>
+        <v>-0.0609011067201433</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>4540</v>
+        <v>4414</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>全球傳動</t>
+          <t>如興</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>274.4322725985672</v>
+        <v>303.0777965631694</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>56.7</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,13 +3414,13 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>39.15815070871226</v>
+        <v>46.29764193570838</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>16.08738664773016</v>
+        <v>16.83253887990648</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.5450606257931619</v>
+        <v>0.4623435669650748</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.7312092506292935</v>
+        <v>0.06304644204970471</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>5515</v>
+        <v>4583</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>建國</t>
+          <t>台灣精銳</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>262.8514640218363</v>
+        <v>291.0945889811774</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>40.45</v>
+        <v>605</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>44.09525901793464</v>
+        <v>38.27581033002252</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>19.73877929943082</v>
+        <v>36.05056018009433</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.4375240452751367</v>
+        <v>0.9339098843506094</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.3100135923285382</v>
+        <v>-0.4191200266180388</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4552</v>
+        <v>4766</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>力達-KY</t>
+          <t>南寶</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>259.380404991768</v>
+        <v>275.5298205404143</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>20.05</v>
+        <v>356.5</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>38.88623204562485</v>
+        <v>48.66618856689502</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>26.4270075343395</v>
+        <v>16.95375094222679</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.7894756094374624</v>
+        <v>1.068839097627098</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.1580525269769042</v>
+        <v>-2.089189099028857</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>4930</v>
+        <v>4540</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>燦星網</t>
+          <t>全球傳動</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>250.7119905683607</v>
+        <v>274.4322725985672</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>16.85</v>
+        <v>56.7</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>36.72595988763544</v>
+        <v>39.15815070871226</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>30.12625354116836</v>
+        <v>16.08738664773016</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>1.229296178584576</v>
+        <v>0.5450606257931619</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0410470227661827</v>
+        <v>-0.7312092506292935</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>5531</v>
+        <v>5515</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>鄉林</t>
+          <t>建國</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>247.178371000491</v>
+        <v>262.8514640218363</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>7.87</v>
+        <v>40.45</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>43.06430467898355</v>
+        <v>44.09525901793464</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>24.1055663289943</v>
+        <v>19.73877929943082</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>0.5761878558548279</v>
+        <v>0.4375240452751367</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.0193157165842924</v>
+        <v>-0.3100135923285382</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4438</v>
+        <v>4552</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>廣越</t>
+          <t>力達-KY</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>242.6298801881052</v>
+        <v>259.380404991768</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>59.3</v>
+        <v>20.05</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>46.21235736052003</v>
+        <v>38.88623204562485</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>24.57725613333918</v>
+        <v>26.4270075343395</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.4513949196360851</v>
+        <v>0.7894756094374624</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.3267004685707815</v>
+        <v>-0.1580525269769042</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4557</v>
+        <v>4930</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>永新-KY</t>
+          <t>燦星網</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>221.2108386984668</v>
+        <v>250.7119905683607</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>47.55</v>
+        <v>16.85</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>49.18762248269263</v>
+        <v>36.72595988763544</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>18.13222993931328</v>
+        <v>30.12625354116836</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.5975849889286453</v>
+        <v>1.229296178584576</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.1500619574096165</v>
+        <v>-0.0410470227661827</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>4440</v>
+        <v>5531</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>宜新實業</t>
+          <t>鄉林</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>212.4897609680073</v>
+        <v>247.178371000491</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>17.15</v>
+        <v>7.87</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>42.00213311914128</v>
+        <v>43.06430467898355</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>14.67723193235939</v>
+        <v>24.1055663289943</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.338696620212976</v>
+        <v>0.5761878558548279</v>
       </c>
       <c r="K63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0110256867452116</v>
+        <v>-0.0193157165842924</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6150</v>
+        <v>4438</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>撼訊</t>
+          <t>廣越</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>211.7895055033156</v>
+        <v>242.6298801881052</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>61</v>
+        <v>59.3</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,13 +3838,13 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>41.91973073004908</v>
+        <v>46.21235736052003</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>17.86201074656555</v>
+        <v>24.57725613333918</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.2796035175564137</v>
+        <v>0.4513949196360851</v>
       </c>
       <c r="K64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.4382485432117672</v>
+        <v>-0.3267004685707815</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>5906</v>
+        <v>4557</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>台南-KY</t>
+          <t>永新-KY</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>208.3016886590108</v>
+        <v>221.2108386984668</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>38</v>
+        <v>47.55</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>51.69522159480197</v>
+        <v>49.18762248269263</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>6.23807096586794</v>
+        <v>18.13222993931328</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.2902408701851938</v>
+        <v>0.5975849889286453</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>1.065557967387386</v>
+        <v>0.1500619574096165</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>4770</v>
+        <v>4440</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>上品</t>
+          <t>宜新實業</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>204.8821280685517</v>
+        <v>212.4897609680073</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>214.5</v>
+        <v>17.15</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>40.46673310282695</v>
+        <v>42.00213311914128</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>21.58493918443004</v>
+        <v>14.67723193235939</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.4951980892431528</v>
+        <v>0.338696620212976</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0058032314727825</v>
+        <v>0.0110256867452116</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>5521</v>
+        <v>6150</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>工信</t>
+          <t>撼訊</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>203.947961784609</v>
+        <v>211.7895055033156</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>10.25</v>
+        <v>61</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>43.51409926245679</v>
+        <v>41.91973073004908</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>17.40019631013624</v>
+        <v>17.86201074656555</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.4730688339208276</v>
+        <v>0.2796035175564137</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0200168894146366</v>
+        <v>-0.4382485432117672</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6151</v>
+        <v>5906</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>晉倫</t>
+          <t>台南-KY</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>201.9117451102081</v>
+        <v>208.3016886590108</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>39.1</v>
+        <v>38</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,13 +4050,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>43.42667237927903</v>
+        <v>51.69522159480197</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>19.81312915591589</v>
+        <v>6.23807096586794</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.3755130264854425</v>
+        <v>0.2902408701851938</v>
       </c>
       <c r="K68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.4425212257215641</v>
+        <v>1.065557967387386</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>5706</v>
+        <v>4770</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>鳳凰</t>
+          <t>上品</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>200.7835105786564</v>
+        <v>204.8821280685517</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>46.95</v>
+        <v>214.5</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>25.93661857835919</v>
+        <v>40.46673310282695</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>25.212220299951</v>
+        <v>21.58493918443004</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.4783510578656386</v>
+        <v>0.4951980892431528</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.7894936669375348</v>
+        <v>-0.0058032314727825</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6158</v>
+        <v>5521</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>禾昌</t>
+          <t>工信</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>188.5731487465727</v>
+        <v>203.947961784609</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>17.25</v>
+        <v>10.25</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>37.5377061695421</v>
+        <v>43.51409926245679</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>25.14734820071165</v>
+        <v>17.40019631013624</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.2979396484721218</v>
+        <v>0.4730688339208276</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.0161739190252152</v>
+        <v>0.0200168894146366</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>4195</v>
+        <v>6151</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>基米-創</t>
+          <t>晉倫</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>187.691613392004</v>
+        <v>201.9117451102081</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>15.4</v>
+        <v>39.1</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>29.9936964383329</v>
+        <v>43.42667237927903</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>41.64125880612912</v>
+        <v>19.81312915591589</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.4278361731509588</v>
+        <v>0.3755130264854425</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.2905525734868281</v>
+        <v>-0.4425212257215641</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>4566</v>
+        <v>5706</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>時碩工業</t>
+          <t>鳳凰</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>173.6633665508131</v>
+        <v>200.7835105786564</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>62</v>
+        <v>46.95</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>45.80157169786316</v>
+        <v>25.93661857835919</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>9.848050519382053</v>
+        <v>25.212220299951</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.4914844589322523</v>
+        <v>0.4783510578656386</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.2005990177958769</v>
+        <v>-0.7894936669375348</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>5608</v>
+        <v>6158</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>四維航</t>
+          <t>禾昌</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>166.5915098643413</v>
+        <v>188.5731487465727</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>14.25</v>
+        <v>17.25</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>40.19503845897982</v>
+        <v>37.5377061695421</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.59038008532424</v>
+        <v>25.14734820071165</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.7093873487806098</v>
+        <v>0.2979396484721218</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.0603310651551983</v>
+        <v>-0.0161739190252152</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>5007</v>
+        <v>4195</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>三星</t>
+          <t>基米-創</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>160.4505742529941</v>
+        <v>187.691613392004</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>56</v>
+        <v>15.4</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.5897816962023</v>
+        <v>29.9936964383329</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>16.18444056696606</v>
+        <v>41.64125880612912</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.232551795551275</v>
+        <v>0.4278361731509588</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.0059904157688841</v>
+        <v>0.2905525734868281</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>5533</v>
+        <v>4566</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>皇鼎</t>
+          <t>時碩工業</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>149.2456152243156</v>
+        <v>173.6633665508131</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>49.79200641934032</v>
+        <v>45.80157169786316</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>15.56986580405409</v>
+        <v>9.848050519382053</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.8631179514918085</v>
+        <v>0.4914844589322523</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0074456616660635</v>
+        <v>-0.2005990177958769</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>5907</v>
+        <v>5608</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>大洋-KY</t>
+          <t>四維航</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>138.7029263655118</v>
+        <v>166.5915098643413</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>4.83</v>
+        <v>14.25</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>36.12961630049733</v>
+        <v>40.19503845897982</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>17.92346249474726</v>
+        <v>15.59038008532424</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.359791978561665</v>
+        <v>0.7093873487806098</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0180359217956542</v>
+        <v>-0.0603310651551983</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4502,21 +4502,21 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6160</v>
+        <v>5007</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>欣技</t>
+          <t>三星</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>95.28732364993834</v>
+        <v>160.4505742529941</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>16.15</v>
+        <v>56</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>43.39701758526012</v>
+        <v>44.5897816962023</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>15.73223308223666</v>
+        <v>16.18444056696606</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.8679629898911562</v>
+        <v>0.232551795551275</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.0938878948965008</v>
+        <v>-0.0059904157688841</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>4426</v>
+        <v>5533</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>利勤</t>
+          <t>皇鼎</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>92.23344266370042</v>
+        <v>149.2456152243156</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>7.93</v>
+        <v>14</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>49.12146514660179</v>
+        <v>49.79200641934032</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>15.21279333819073</v>
+        <v>15.56986580405409</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.5055968973843565</v>
+        <v>0.8631179514918085</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0048181388643404</v>
+        <v>0.0074456616660635</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4608,21 +4608,21 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>4562</v>
+        <v>5907</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>穎漢</t>
+          <t>大洋-KY</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>71.08309928851509</v>
+        <v>138.7029263655118</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>33.7</v>
+        <v>4.83</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>39.42080801400962</v>
+        <v>36.12961630049733</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>16.8078837757534</v>
+        <v>17.92346249474726</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.4563037345928901</v>
+        <v>0.359791978561665</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.3316663010559839</v>
+        <v>-0.0180359217956542</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4661,21 +4661,21 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>4736</v>
+        <v>6160</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>泰博</t>
+          <t>欣技</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>70.32766894256346</v>
+        <v>95.28732364993834</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>123.5</v>
+        <v>16.15</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>46.69013259488972</v>
+        <v>43.39701758526012</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>17.66704968918249</v>
+        <v>15.73223308223666</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.6012534792451936</v>
+        <v>0.8679629898911562</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.137933987677359</v>
+        <v>-0.0938878948965008</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,52 +4714,211 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
+        <v>4426</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>利勤</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>92.23344266370042</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H81" s="2" t="n">
+        <v>49.12146514660179</v>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>15.21279333819073</v>
+      </c>
+      <c r="J81" s="2" t="n">
+        <v>0.5055968973843565</v>
+      </c>
+      <c r="K81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N81" s="2" t="n">
+        <v>-0.0048181388643404</v>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>4562</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>穎漢</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>71.08309928851509</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H82" s="2" t="n">
+        <v>39.42080801400962</v>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>16.8078837757534</v>
+      </c>
+      <c r="J82" s="2" t="n">
+        <v>0.4563037345928901</v>
+      </c>
+      <c r="K82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N82" s="2" t="n">
+        <v>-0.3316663010559839</v>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>4736</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>泰博</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>70.32766894256346</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>46.69013259488972</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>17.66704968918249</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.6012534792451936</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>-0.137933987677359</v>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
         <v>4441</v>
       </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>振大環球</t>
         </is>
       </c>
-      <c r="C81" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D81" s="2" t="n">
+      <c r="C84" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D84" s="2" t="n">
         <v>60.70092593400895</v>
       </c>
-      <c r="E81" s="2" t="n">
+      <c r="E84" s="2" t="n">
         <v>191.5</v>
       </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H81" s="2" t="n">
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
         <v>43.85303711772298</v>
       </c>
-      <c r="I81" s="2" t="n">
+      <c r="I84" s="2" t="n">
         <v>13.36678914829477</v>
       </c>
-      <c r="J81" s="2" t="n">
+      <c r="J84" s="2" t="n">
         <v>0.6533509372694614</v>
       </c>
-      <c r="K81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L81" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M81" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N81" s="2" t="n">
+      <c r="K84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N84" s="2" t="n">
         <v>-1.085726604866848</v>
       </c>
-      <c r="O81" s="2" t="inlineStr">
+      <c r="O84" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>